<commit_message>
fix(curriculum): lộ trình theo template — Mục tiêu + BT về nhà cho 32 buổi
User feedback: muốn format giáo án rõ 2 phần cho mỗi buổi:
1. Mục tiêu — học viên được dạy gì hôm đó
2. BT về nhà — nộp gì, coi gì trước cho buổi sau

Bỏ cột 'Nội dung chính (vắn tắt)' (trùng với Mục tiêu).

Sheet 'Lộ trình' giờ có 8 cột:
  Buổi | Tuần | Tháng | Chủ đề | Mục tiêu buổi học | Bài tập về nhà | Theme | Bài tập map

Mỗi cell Mục tiêu / BT về nhà = bullet points (xuống dòng \\n trong cell).
Width tối ưu: Mục tiêu 70 ký tự, BT về nhà 70 ký tự.
Row height 130 cho cell render đủ multi-line.
Freeze pane + auto filter ở header.

Mỗi buổi BT về nhà có 3 phần (theo template Doc gốc):
  • Nộp: <bài tập cụ thể>
  • Coi trước: <prep cho buổi sau>
  • (optional) Chuẩn bị: <slide / setup>

Output:
  docs/giao_an_hoc_vien.xlsx           34 KB (5 sheets)
  docs/giao_an_hoc_vien_csv/lo_trinh.csv  33 dòng (1 header + 32 buổi)
</commit_message>
<xml_diff>
--- a/docs/giao_an_hoc_vien.xlsx
+++ b/docs/giao_an_hoc_vien.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Hướng dẫn" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lộ trình'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bài tập'!$A$1:$J$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -719,17 +720,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Buổi</t>
@@ -737,826 +741,1360 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>Tuần</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Tháng</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Chủ đề</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Nội dung chính (vắn tắt)</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Mục tiêu buổi học</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Bài tập về nhà</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Bài tập</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="60" customHeight="1">
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Bài tập map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="130" customHeight="1">
       <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 1 — Intro tool + dataset Shopee</t>
-        </is>
+      <c r="B2" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Setup tool, đăng nhập, schema fact/dim, SELECT/FROM/WHERE/LIMIT, đọc số top-line: COUNT đơn, SUM total_amount.</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
+          <t>Intro tool + dataset Shopee + SELECT cơ bản</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>• Đăng nhập tool, làm quen UI (editor, schema browser, kết quả).
+• Hiểu cấu trúc schema 'shopee' — phân biệt bảng fact (giao dịch) vs dim (master).
+• Viết SELECT đơn giản với FROM, WHERE, LIMIT.
+• Đọc số top-line cơ bản: COUNT(*) số đơn, SUM(total_amount) doanh thu.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: viết 5 query SELECT trên fact_orders với filter khác nhau (status, payment_method, ngày).
+• Coi trước: sheet 'Schema' — đọc kỹ dim_date, dim_customer, dim_product.
+• Chuẩn bị: ghi chú 3 câu hỏi business muốn trả lời từ dataset.</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="130" customHeight="1">
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 2 — ORDER BY, DISTINCT, operators</t>
-        </is>
+      <c r="B3" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>ORDER BY ASC/DESC, DISTINCT, IN/BETWEEN/LIKE/IS NULL, string functions cơ bản (LOWER, UPPER, TRIM, ||).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
+          <t>ORDER BY, DISTINCT, operators</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>• Sort kết quả với ORDER BY ASC/DESC, sort theo nhiều cột.
+• Loại trùng với DISTINCT, COUNT(DISTINCT col).
+• Dùng các operator: IN, BETWEEN, LIKE, IS NULL.
+• String functions cơ bản: LOWER, UPPER, TRIM, concat ||.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: list top 20 đơn cao nhất theo total_amount.
+• Nộp: list distinct payment_method và số đơn mỗi loại.
+• Nộp: tìm shop có shop_name chứa từ 'Store' (case-insensitive).
+• Coi trước: khái niệm aggregate (COUNT, SUM, AVG, MIN, MAX).</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>(luyện cú pháp)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="130" customHeight="1">
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 3 — Aggregate functions</t>
-        </is>
+      <c r="B4" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>COUNT, SUM, AVG, MIN, MAX, COUNT(DISTINCT). Tính GMV, AOV, basket size. Phân biệt COUNT(*) vs COUNT(col).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
+          <t>Aggregate functions</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>• Phân biệt COUNT(*), COUNT(col), COUNT(DISTINCT col).
+• Tính GMV (SUM total_amount), AOV (SUM/COUNT), max/min order.
+• Hiểu khi nào dùng aggregate function nào cho metric biz.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài A1, A2 (sheet Bài tập). Lưu ý filter payment_status='paid' khi tính GMV.
+• Coi trước: GROUP BY là gì, vì sao cần?</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>A1, A2</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="130" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 4 — GROUP BY + HAVING</t>
-        </is>
+      <c r="B5" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>GROUP BY 1 cột, nhiều cột. HAVING vs WHERE. GMV theo ngày/tuần/tháng (DATE_TRUNC sơ lược).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
+          <t>GROUP BY + HAVING</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>• GROUP BY 1 cột rồi nhiều cột.
+• Phân biệt HAVING vs WHERE (filter trước/sau aggregate).
+• GMV theo ngày/tuần/tháng — sơ lược DATE_TRUNC.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài A3, A4.
+• Coi trước: khái niệm JOIN — vì sao cần JOIN nhiều bảng?</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>A3, A4</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="130" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 5 — INNER JOIN</t>
-        </is>
+      <c r="B6" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Khái niệm join, JOIN 2 bảng (fact_orders + dim_date), JOIN 3 bảng (orders + items + product).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>INNER JOIN</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>• Hiểu join là gì, vẽ Venn diagram.
+• JOIN 2 bảng (fact_orders + dim_date), 3 bảng (orders + items + product).
+• Dùng alias cho dễ đọc; ON condition đúng khoá.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài A5 (GMV theo cat1), Bài F1.
+• Coi trước: LEFT JOIN khác INNER chỗ nào? Khi nào cần LEFT?</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>A, F</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>A5, F1</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="130" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 6 — LEFT/RIGHT/FULL JOIN</t>
-        </is>
+      <c r="B7" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Khi nào dùng LEFT vs INNER. Tìm 'customer chưa mua', 'sản phẩm chưa bán'. Anti-join pattern (NOT EXISTS / LEFT IS NULL).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
+          <t>LEFT / RIGHT / FULL JOIN</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>• Khi nào dùng LEFT vs INNER. NULL từ bên không match.
+• Anti-join pattern: customer chưa từng mua, sản phẩm chưa bán.
+• LEFT JOIN ... WHERE x IS NULL = NOT EXISTS.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài B1 (customer chưa quay lại), Bài F2 (sản phẩm bán chậm).
+• Coi trước: query 5+ bảng — chiến lược tránh nhầm Cartesian.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
           <t>B, F</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>B1, F2</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="130" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 7 — Multi-table JOIN nâng cao</t>
-        </is>
+      <c r="B8" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>JOIN 4-5 bảng. Bí quyết tránh Cartesian. Alias rõ ràng. Decompose query phức tạp.</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
+          <t>Multi-table JOIN nâng cao</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>• JOIN 4-5 bảng trong 1 query, alias rõ ràng.
+• Decompose query phức tạp thành step nhỏ.
+• Phát hiện + tránh Cartesian product (cardinality check).</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài F3 (top SP theo cat), Bài K1 (GMV theo region).
+• Chuẩn bị mini-project tháng 1: GMV weekly report.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
           <t>F, K</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>F3, K1</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="130" customHeight="1">
       <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 8 — Mini-project tháng 1</t>
-        </is>
+      <c r="B9" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Bài tổng hợp: viết GMV weekly report đầy đủ với MoM growth. Trình bày trên Google Sheets (paste TSV từ tool).</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
+          <t>Mini-project tháng 1: GMV Weekly Report</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>• Tổng hợp SQL foundation đã học.
+• Viết end-to-end report GMV weekly với MoM growth.
+• Trình bày kết quả Google Sheets (paste TSV từ tool).</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: 1 query SQL + 1 trang Google Sheets phân tích insights.
+• Coi trước: DATE_TRUNC, EXTRACT — chuẩn bị cho tháng 2.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>A6, A7, A8</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="130" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 9 — DATE_TRUNC, EXTRACT, INTERVAL</t>
-        </is>
+      <c r="B10" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>DATE_TRUNC('week'/'month'/'quarter'). EXTRACT(DOW/HOUR). INTERVAL math. Pattern theo giờ trong ngày.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
+          <t>DATE_TRUNC, EXTRACT, INTERVAL</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>• DATE_TRUNC ('day', 'week', 'month', 'quarter') — group theo period.
+• EXTRACT (DOW, HOUR, MONTH) — bóc thành phần.
+• INTERVAL math: cộng/trừ ngày, tính tuổi đơn.
+• Pattern theo giờ trong ngày: peak hour, dip hour.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài C1 (GMV theo giờ), C2 (GMV theo ngày trong tuần).
+• Coi trước: WoW / MoM growth — cách so sánh kỳ với kỳ.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>C1, C2</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="130" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 10 — Time-series: WoW, MoM, YoY</t>
-        </is>
+      <c r="B11" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>So sánh kỳ với kỳ. Self-join trên dim_date (chưa dùng window). Tăng trưởng tuyệt đối vs tăng trưởng %.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
+          <t>Time-series: WoW, MoM, YoY growth</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>• So sánh tuần này vs tuần trước (WoW), tháng vs tháng trước (MoM).
+• Self-join trên dim_date để align period.
+• Tăng trưởng tuyệt đối (Δ) vs tăng trưởng % (growth rate).</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài C3, C4.
+• Coi trước: subquery — query lồng nhau, IN / EXISTS.</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>C3, C4</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="130" customHeight="1">
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 11 — Subquery cơ bản</t>
-        </is>
+      <c r="B12" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Scalar subquery, subquery trong WHERE/IN/EXISTS. Khi nào nên dùng subquery vs JOIN.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>Subquery cơ bản</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>• Scalar subquery (trả 1 giá trị).
+• Subquery trong WHERE: IN, NOT IN, EXISTS, NOT EXISTS.
+• Khi nào nên dùng subquery vs JOIN — trade-off readability vs performance.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài B2 (customer mua &gt; X đơn), F4 (sản phẩm có rating cao).
+• Coi trước: CTE (WITH clause) — vì sao CTE tốt hơn nested subquery?</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>B, F</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>B2, F4</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="130" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 12 — CTE (WITH clause)</t>
-        </is>
+      <c r="B13" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>WITH ... AS (...) SELECT. Multi-CTE. Lý do CTE &gt; nested subquery: dễ đọc, dễ debug.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>CTE — WITH clause</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>• Cú pháp WITH name AS (...) SELECT.
+• Multi-CTE: WITH a AS (...), b AS (...) — chain logic.
+• Lợi: dễ đọc, dễ debug, có thể reference nhiều lần.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài B3 (segment customer), B4 (cohort signup theo tháng).
+• Coi trước: window function là gì? Khác aggregate chỗ nào?</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>B3, B4</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="130" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 13 — Window function intro</t>
-        </is>
+      <c r="B14" s="5" t="n">
+        <v>7</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>OVER (), PARTITION BY, ORDER BY trong window. Khác biệt aggregate vs window aggregate (giữ nguyên row).</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
+          <t>Window function intro: OVER, PARTITION BY</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>• Khái niệm window: aggregate KHÔNG collapse row.
+• OVER (PARTITION BY ... ORDER BY ...) — khung tính toán.
+• Use case: % share trong group, rank trong group.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài F5 (% GMV mỗi cat trong tổng).
+• Coi trước: ROW_NUMBER, RANK, DENSE_RANK — khác nhau ra sao?</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>F5</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="130" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 14 — Ranking: ROW_NUMBER, RANK, NTILE</t>
-        </is>
+      <c r="B15" s="5" t="n">
+        <v>7</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Top-N per group (top 5 SP mỗi seller). RANK vs DENSE_RANK. NTILE để chia tier (RFM segment).</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
+          <t>Ranking: ROW_NUMBER, RANK, DENSE_RANK, NTILE</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>• ROW_NUMBER vs RANK vs DENSE_RANK — handle ties.
+• Top-N per group (top 5 SP mỗi seller).
+• NTILE để chia tier (RFM: 5 nhóm Recency/Frequency/Monetary).</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài F6 (top 5 SP mỗi seller), B5 (xếp tier customer).
+• Coi trước: LAG, LEAD — tính growth rate qua window.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
           <t>F, B</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>F6, B5</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="130" customHeight="1">
       <c r="A16" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 15 — LAG, LEAD, running total</t>
-        </is>
+      <c r="B16" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Lag để tính growth %. Lead để check next event. SUM(...) OVER (ORDER BY ... ROWS BETWEEN ...) cho running total/MA.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
+          <t>LAG, LEAD, running total, moving average</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>• LAG để tính growth %: (this - prev) / prev.
+• LEAD để check next event (next purchase, next session).
+• SUM(...) OVER (ORDER BY ... ROWS BETWEEN ...) cho running total / MA-7.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài A8 extension (MoM growth qua LAG), B6 (thời gian giữa 2 đơn).
+• Chuẩn bị mini-project tháng 2: cohort retention.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
           <t>A, B</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>A8 ext, B6</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="130" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 16 — Mini-project tháng 2</t>
-        </is>
+      <c r="B17" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Cohort retention 7/30 ngày + MoM signup growth. Output: bảng cohort matrix.</t>
+          <t>Tháng 2</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
+          <t>Mini-project tháng 2: Cohort retention 7/30</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>• Tổng hợp time + window + CTE.
+• Build cohort matrix: signup_month × tháng quay lại.
+• Tính retention rate 7d / 30d / 90d.</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: 1 query cohort + bảng matrix paste vào Google Sheets.
+• Coi trước: RFM segmentation — recency/frequency/monetary.</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>B7, B8, B9</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="130" customHeight="1">
       <c r="A18" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 17 — RFM customer segmentation</t>
-        </is>
+      <c r="B18" s="5" t="n">
+        <v>9</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Recency / Frequency / Monetary. NTILE chia 5 tier. Crossing 3 dimension → 125 segment (rút gọn còn 4-5 nhóm chính).</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
+          <t>RFM customer segmentation</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>• RFM = Recency × Frequency × Monetary.
+• Dùng NTILE chia 5 tier mỗi dimension → 125 segment.
+• Rút gọn 125 → 4-5 nhóm chính (Champion, Loyal, At-risk, Lost…).</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: query RFM + danh sách 100 'Champion customer' để remarketing.
+• Coi trước: voucher analysis — redemption rate là gì?</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>B (extension)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>(B mở rộng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="130" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 18 — Voucher / promotion analysis</t>
-        </is>
+      <c r="B19" s="5" t="n">
+        <v>9</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Voucher redemption rate, average discount per order. Voucher có thật sự drive incremental orders?</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
+          <t>Voucher / promotion analysis</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>• Voucher redemption rate = (used / issued).
+• Avg discount per order, total discount cost.
+• Voucher có drive incremental orders, hay chỉ subsidize organic?</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài D1, D2, D3, D4.
+• Coi trước: campaign uplift — đo hiệu quả campaign so với baseline.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>D1-D4</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20" ht="130" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 19 — Campaign uplift</t>
-        </is>
+      <c r="B20" s="5" t="n">
+        <v>10</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Compare campaign period vs baseline (3 tuần trước). Cẩn thận seasonality. Self-join hoặc CTE để tính uplift.</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
+          <t>Campaign uplift</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>• Compare campaign period vs baseline (3 tuần trước cùng kỳ).
+• Cẩn thận seasonality, lễ tết.
+• Self-join hoặc CTE để tính uplift %.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài C5, C6, C7, D5, D6, D7.
+• Coi trước: ROAS = Return on Ad Spend, CTR, CPC.</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
           <t>C, D</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>C5-C7, D5-D7</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21" ht="130" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 20 — Marketing: ROAS, CTR, CPC</t>
-        </is>
+      <c r="B21" s="5" t="n">
+        <v>10</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>fact_ad_spend × fact_ad_performance_daily. Tính ROAS, CTR, CPC theo channel/campaign. Channel nào hiệu quả nhất?</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
+          <t>Marketing: ROAS, CTR, CPC</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>• JOIN fact_ad_spend × fact_ad_performance_daily.
+• Tính ROAS (revenue/spend), CTR (clicks/impressions), CPC (spend/clicks).
+• So sánh hiệu quả channel: search vs display vs affiliate vs KOL.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài G1, G2, G3, G4.
+• Coi trước: seller performance — long tail vs head sellers.</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
           <t>G</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>G1-G4</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="130" customHeight="1">
       <c r="A22" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 21 — Seller performance</t>
-        </is>
+      <c r="B22" s="5" t="n">
+        <v>11</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Top sellers theo GMV/units/AOV. Long tail vs head. Shop_type (mall/preferred/normal) ảnh hưởng GMV?</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
+          <t>Seller performance</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>• Top sellers theo GMV / units sold / AOV.
+• Pareto 80/20: top 20% sellers chiếm bao nhiêu % GMV?
+• Shop_type (mall / preferred / normal) ảnh hưởng GMV / cancel rate?</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài E1, E2, E3, E4.
+• Coi trước: product / category trends — cat nào growth nhất?</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
           <t>E</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>E1-E4</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="130" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 22 — Product / category trends</t>
-        </is>
+      <c r="B23" s="5" t="n">
+        <v>11</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Cat1 nào growth nhất 3 tháng qua? Brand contribution. Pareto 80/20 trên SKU level.</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
+          <t>Product / Category trends</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>• Cat1 nào growth GMV nhanh nhất 3 tháng qua?
+• Brand contribution: top brand mỗi cat1.
+• Pareto trên SKU level — 20% SKU sinh 80% GMV?</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài F7, F8.
+• Coi trước: geographic analysis — region/province.</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
           <t>F</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>F7, F8</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24" ht="130" customHeight="1">
       <c r="A24" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 23 — Geographic analysis</t>
-        </is>
+      <c r="B24" s="5" t="n">
+        <v>12</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>GMV theo region (north/central/south). Penetration rate. Province nào tỷ lệ cancel cao bất thường?</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
+          <t>Geographic analysis</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>• GMV theo region (north/central/south).
+• Penetration rate: % customer / population (giả định population).
+• Province nào tỷ lệ cancel cao bất thường? (red flag).</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài K1, K2, K3, K4, K5.
+• Chuẩn bị mini-project tháng 3: marketing dashboard.</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>K1-K5</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25" ht="130" customHeight="1">
       <c r="A25" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 24 — Mini-project tháng 3</t>
-        </is>
+      <c r="B25" s="5" t="n">
+        <v>12</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Marketing dashboard end-to-end: top campaign, top seller, top SKU, ROAS theo channel. Trình bày bằng số + chart suggestion.</t>
+          <t>Tháng 3</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
+          <t>Mini-project tháng 3: Marketing Dashboard</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>• Tổng hợp business analytics đã học.
+• Build dashboard: top campaign, top seller, top SKU, ROAS theo channel.
+• Trình bày bằng số + chart suggestion (loại chart nào cho metric nào).</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Google Sheets dashboard 1 trang + insight 3-5 bullet.
+• Coi trước: shipping &amp; SLA — on-time rate là gì.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
           <t>C, D, E, G</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>(tổng hợp)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="130" customHeight="1">
       <c r="A26" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 25 — Shipping &amp; SLA</t>
-        </is>
+      <c r="B26" s="5" t="n">
+        <v>13</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>On-time delivery rate. SLA breach theo carrier/route. Avg delivery time intra-city vs cross-region.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
+          <t>Shipping &amp; SLA analysis</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>• On-time delivery rate = is_on_time / total shipments.
+• SLA breach theo carrier, theo route (intra-city / cross-region).
+• Avg delivery time + p90/p95.</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài H1, H2, H3, H4.
+• Coi trước: cancel/return analysis — pattern lý do hủy.</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
           <t>H</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>H1-H4</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27" ht="130" customHeight="1">
       <c r="A27" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 26 — Cancellation &amp; return</t>
-        </is>
+      <c r="B27" s="5" t="n">
+        <v>13</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Cancel rate theo lý do, theo seller. Return reason analysis. Buyer cancel vs seller cancel patterns.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
+          <t>Cancellation &amp; return analysis</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>• Cancel rate theo lý do, theo seller, theo cat1.
+• Return reason analysis — top 3 lý do return.
+• Buyer cancel (customer_change_mind) vs seller cancel (out_of_stock) — phân biệt.</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài I1, I2, I3, I4.
+• Coi trước: customer service tickets — category breakdown.</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
           <t>I</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>I1-I4</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
+    <row r="28" ht="130" customHeight="1">
       <c r="A28" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 27 — Customer service tickets</t>
-        </is>
+      <c r="B28" s="5" t="n">
+        <v>14</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Ticket category distribution. Avg resolution time. Seller nào nhiều complaint nhất? Correlation với cancel/return.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
+          <t>Customer service tickets</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>• Ticket category distribution: shipping vs quality vs refund.
+• Avg resolution time (resolved_at - created_at).
+• Seller nào nhiều complaint nhất — correlation với cancel/return.</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài J1, J2, J3, J4, J5.
+• Coi trước: advanced patterns — FILTER, conditional aggregate.</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
           <t>J</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>J1-J5</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1">
+    <row r="29" ht="130" customHeight="1">
       <c r="A29" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 28 — Advanced SQL patterns</t>
-        </is>
+      <c r="B29" s="5" t="n">
+        <v>14</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>FILTER (WHERE ...), conditional aggregate, PIVOT bằng FILTER. CASE WHEN trong aggregate. JSON functions (nếu có thời gian).</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>L (intro)</t>
+          <t>Advanced SQL patterns</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
+          <t>• FILTER (WHERE ...) trong aggregate — pivot bằng FILTER.
+• CASE WHEN trong SUM/COUNT để conditional metric.
+• Cú pháp pivot manual: SUM(CASE WHEN cat='X' THEN ...) AS x_gmv.</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Bài L1, L2 (capstone — chuẩn bị).
+• Coi trước: EXPLAIN — đọc execution plan cơ bản.</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
           <t>L1, L2</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30" ht="130" customHeight="1">
       <c r="A30" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 29 — Performance &amp; EXPLAIN</t>
-        </is>
+      <c r="B30" s="5" t="n">
+        <v>15</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Index, EXPLAIN basic. Vì sao query chậm? Best practice: filter sớm, tránh SELECT *, JOIN order.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
+          <t>Performance &amp; EXPLAIN</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>• EXPLAIN cơ bản — đọc plan output.
+• Vì sao query chậm: full scan, missing index, bad join order.
+• Best practice: filter sớm, tránh SELECT *, dùng index column trong WHERE.</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: 3 query đã optimize (kèm EXPLAIN trước/sau).
+• Bốc 1 case study từ theme L cho capstone (sẽ làm 2 buổi).</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>(thực hành EXPLAIN)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31" ht="130" customHeight="1">
       <c r="A31" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 30 — Capstone phần 1</t>
-        </is>
+      <c r="B31" s="5" t="n">
+        <v>15</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Bốc 1 case business thật từ theme L. Định nghĩa câu hỏi, phân rã thành sub-query, viết draft.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
+          <t>Capstone — Phần 1: phân rã &amp; draft query</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>• Định nghĩa câu hỏi business của capstone.
+• Phân rã thành 3-5 sub-question.
+• Viết draft SQL cho từng sub-question.</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: outline capstone + draft query (chưa cần hoàn thiện).
+• Coi trước: cách viết insight + recommendation.</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>L3-L8 (tự chọn)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="60" customHeight="1">
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>L3-L8 (tự chọn 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="130" customHeight="1">
       <c r="A32" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 31 — Capstone phần 2</t>
-        </is>
+      <c r="B32" s="5" t="n">
+        <v>16</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Hoàn thiện query, validate kết quả, viết insight + recommendation. Format Google Slides / Sheets.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
+          <t>Capstone — Phần 2: hoàn thiện + viết insight</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>• Validate kết quả query: cross-check số, edge case.
+• Viết insight (số nói gì) + recommendation (nên làm gì).
+• Format slide / Sheets cho final presentation.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>• Nộp: Google Slides / Sheets capstone hoàn chỉnh (5-7 slide).
+• Chuẩn bị: trình bày 5-7 phút buổi sau.</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>L9-L14</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1">
+    <row r="33" ht="130" customHeight="1">
       <c r="A33" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Buổi 32 — Final presentation + Q&amp;A</t>
-        </is>
+      <c r="B33" s="5" t="n">
+        <v>16</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Mỗi học viên trình bày capstone 5-7 phút. Giảng viên + bạn cùng lớp feedback. Tổng kết khoá + roadmap nâng cao.</t>
+          <t>Tháng 4</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
+          <t>Final presentation + Q&amp;A + Tổng kết khoá</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>• Mỗi học viên trình bày capstone 5-7 phút.
+• Q&amp;A từ giảng viên + bạn cùng lớp.
+• Tổng kết: skill đã học, roadmap nâng cao (analytics engineer, BI dev).</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>• Final: bản capstone v2 (sau feedback).
+• Roadmap nâng cao: học dbt, đọc 'SQL for Data Analysts' (Cathy Tanimura).</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>L15-L17</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>